<commit_message>
Before start of bqr scripting 1
</commit_message>
<xml_diff>
--- a/DataProvider/TestCases_SurfaceUI.xlsx
+++ b/DataProvider/TestCases_SurfaceUI.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="11">
   <si>
     <t xml:space="preserve">Test Case ID</t>
   </si>
@@ -48,6 +48,9 @@
   </si>
   <si>
     <t xml:space="preserve">test_GUI_APP_Branding_Axis_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">False</t>
   </si>
   <si>
     <t xml:space="preserve">test_GUI_APP_Branding_Hdfc_03</t>
@@ -256,7 +259,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultColWidth="11.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="39.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="77.2"/>
@@ -302,12 +305,12 @@
         <v>6</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>5</v>
@@ -316,7 +319,7 @@
         <v>6</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -342,7 +345,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="11.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>